<commit_message>
chore: regenerate vendored artifacts and previews from current builders
The committed Office files and their preview PNGs predated the copy
waves: the binaries carried 8 instances of the removed screening term
and 49 em-dashes, and the in-app preview rail rendered those stale
pages. Rebuilt all three artifacts and re-rendered every preview from
the current builders (all clean). The render script's module hooks now
attach the json import attribute plain node requires, it had been
broken since the model engine gained its static data import.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/artifacts/jahez-valuation-model.xlsx
+++ b/public/artifacts/jahez-valuation-model.xlsx
@@ -12,7 +12,7 @@
     <sheet sheetId="6" name="Sensitivity" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Comps" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Scenarios &amp; Risk" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Shariah Screen" state="visible" r:id="rId12"/>
+    <sheet sheetId="9" name="Compliance Screen" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -28,7 +28,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.2
-Open in Faheem — faheem://doc/market-data-comps/2</t>
+Open in Faheem, faheem://doc/market-data-comps/2</t>
         </r>
       </text>
     </comment>
@@ -36,7 +36,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.2
-Open in Faheem — faheem://doc/market-data-comps/2</t>
+Open in Faheem, faheem://doc/market-data-comps/2</t>
         </r>
       </text>
     </comment>
@@ -44,7 +44,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.3
-Open in Faheem — faheem://doc/market-data-comps/3</t>
+Open in Faheem, faheem://doc/market-data-comps/3</t>
         </r>
       </text>
     </comment>
@@ -52,7 +52,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.3
-Open in Faheem — faheem://doc/market-data-comps/3</t>
+Open in Faheem, faheem://doc/market-data-comps/3</t>
         </r>
       </text>
     </comment>
@@ -60,29 +60,29 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.3
-Open in Faheem — faheem://doc/market-data-comps/3
-n/a — insufficient trading history (IPO'd Dec 2024)</t>
+Open in Faheem, faheem://doc/market-data-comps/3
+n/a, insufficient trading history (IPO'd Dec 2024)</t>
         </r>
       </text>
     </comment>
     <comment ref="C10" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: levered beta = comp-set median of DoorDash 1.78 and Delivery Hero 1.86 (Talabat n/a — insufficient trading history), per Market Data &amp; Comparables Snapshot p.3. Jahez's own 0.02 5Y beta is a thin-trading artifact and is NOT used. A bottom-up unlever/relever to Jahez's capital structure is the flagged next step.</t>
+          <t>Assumption, analyst judgment: levered beta = comp-set median of DoorDash 1.78 and Delivery Hero 1.86 (Talabat n/a, insufficient trading history), per Market Data &amp; Comparables Snapshot p.3. Jahez's own 0.02 5Y beta is a thin-trading artifact and is NOT used. A bottom-up unlever/relever to Jahez's capital structure is the flagged next step.</t>
         </r>
       </text>
     </comment>
     <comment ref="C12" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: cost-of-debt spread of +200bps over the risk-free rate. No clean Jahez credit spread is sourceable (Cbonds Saudi IG index is paywalled; the sovereign USD spread of ~50–100bps is sovereign, not corporate). 200bps reflects an unrated but cash-generative KSA mid-cap.</t>
+          <t>Assumption, analyst judgment: cost-of-debt spread of +200bps over the risk-free rate. No clean Jahez credit spread is sourceable (Cbonds Saudi IG index is paywalled; the sovereign USD spread of ~50–100bps is sovereign, not corporate). 200bps reflects an unrated but cash-generative KSA mid-cap.</t>
         </r>
       </text>
     </comment>
     <comment ref="C14" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: Saudi zakat convention ~2.5% of the zakat base for Saudi/GCC-owned entities (vs the 20% CIT that applies to foreign ownership). Q1-26 zakat of SAR 0.12m sat on a pre-zakat loss, so no meaningful effective rate is observable. Applied as the NOPAT tax rate and the debt tax-shield.</t>
+          <t>Assumption, analyst judgment: Saudi zakat convention ~2.5% of the zakat base for Saudi/GCC-owned entities (vs the 20% CIT that applies to foreign ownership). Q1-26 zakat of SAR 0.12m sat on a pre-zakat loss, so no meaningful effective rate is observable. Applied as the NOPAT tax rate and the debt tax-shield.</t>
         </r>
       </text>
     </comment>
@@ -90,7 +90,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.24
-Open in Faheem — faheem://doc/q1-26-fs/24
+Open in Faheem, faheem://doc/q1-26-fs/24
 209,836,060 shares at SR 0.5 par (note 9)</t>
         </r>
       </text>
@@ -99,7 +99,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.2
-Open in Faheem — faheem://doc/market-data-comps/2</t>
+Open in Faheem, faheem://doc/market-data-comps/2</t>
         </r>
       </text>
     </comment>
@@ -107,7 +107,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.4
-Open in Faheem — faheem://doc/q1-26-fs/4</t>
+Open in Faheem, faheem://doc/q1-26-fs/4</t>
         </r>
       </text>
     </comment>
@@ -115,7 +115,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.4
-Open in Faheem — faheem://doc/q1-26-fs/4</t>
+Open in Faheem, faheem://doc/q1-26-fs/4</t>
         </r>
       </text>
     </comment>
@@ -123,49 +123,49 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.4
-Open in Faheem — faheem://doc/q1-26-fs/4</t>
+Open in Faheem, faheem://doc/q1-26-fs/4</t>
         </r>
       </text>
     </comment>
     <comment ref="C29" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: long-run nominal terminal growth ~3.0% — broadly Saudi long-term inflation / nominal GDP, below the explicit-period growth and above zero real. Bull 3.5% / Bear 2.5%.</t>
+          <t>Assumption, analyst judgment: long-run nominal terminal growth ~3.0%, broadly Saudi long-term inflation / nominal GDP, below the explicit-period growth and above zero real. Bull 3.5% / Bear 2.5%.</t>
         </r>
       </text>
     </comment>
     <comment ref="C30" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: IRR hold period = 4 years, the mid-point of Lunar's 3–5 year mandate window (see Lunar IC Charter).</t>
+          <t>Assumption, analyst judgment: IRR hold period = 4 years, the mid-point of Lunar's 3–5 year mandate window (see Lunar IC Charter).</t>
         </r>
       </text>
     </comment>
     <comment ref="C31" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: explicit forecast horizon of five years (FY26E–FY30E), then Gordon-growth terminal value.</t>
+          <t>Assumption, analyst judgment: explicit forecast horizon of five years (FY26E–FY30E), then Gordon-growth terminal value.</t>
         </r>
       </text>
     </comment>
     <comment ref="C33" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: D&amp;A held at 3.5% of net revenue (FY25 actual ~3.85%; normalises slightly lower as the IFRS-16 right-of-use base matures).</t>
+          <t>Assumption, analyst judgment: D&amp;A held at 3.5% of net revenue (FY25 actual ~3.85%; normalises slightly lower as the IFRS-16 right-of-use base matures).</t>
         </r>
       </text>
     </comment>
     <comment ref="C34" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: capex at 2.5% of net revenue. No capex line is disclosed in the pack; Jahez is an asset-light platform, so this is set modestly above steady-state maintenance capex.</t>
+          <t>Assumption, analyst judgment: capex at 2.5% of net revenue. No capex line is disclosed in the pack; Jahez is an asset-light platform, so this is set modestly above steady-state maintenance capex.</t>
         </r>
       </text>
     </comment>
     <comment ref="C35" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: ΔNWC drag at 2.0% of the change in net revenue. Delivery platforms run negative-to-near-zero working capital (collect from diners fast, settle restaurants/riders later); a small 2% drag on incremental revenue is deliberately conservative.</t>
+          <t>Assumption, analyst judgment: ΔNWC drag at 2.0% of the change in net revenue. Delivery platforms run negative-to-near-zero working capital (collect from diners fast, settle restaurants/riders later); a small 2% drag on incremental revenue is deliberately conservative.</t>
         </r>
       </text>
     </comment>
@@ -183,7 +183,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.24
-Open in Faheem — faheem://doc/fy24-ar/24</t>
+Open in Faheem, faheem://doc/fy24-ar/24</t>
         </r>
       </text>
     </comment>
@@ -191,7 +191,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -199,42 +199,42 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F5" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
+          <t>Assumption, analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
         </r>
       </text>
     </comment>
     <comment ref="G5" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
+          <t>Assumption, analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
         </r>
       </text>
     </comment>
     <comment ref="H5" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
+          <t>Assumption, analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
         </r>
       </text>
     </comment>
     <comment ref="I5" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
+          <t>Assumption, analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
         </r>
       </text>
     </comment>
     <comment ref="J5" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
+          <t>Assumption, analyst judgment: order growth FY26E +18% (Snoonu full-year consolidation from Oct-2025 plus organic; Q1-26 orders +21% YoY), tapering toward +6% single-market maturity by FY30E.</t>
         </r>
       </text>
     </comment>
@@ -242,7 +242,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.24
-Open in Faheem — faheem://doc/fy24-ar/24</t>
+Open in Faheem, faheem://doc/fy24-ar/24</t>
         </r>
       </text>
     </comment>
@@ -250,7 +250,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -258,42 +258,42 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F7" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
+          <t>Assumption, analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
         </r>
       </text>
     </comment>
     <comment ref="G7" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
+          <t>Assumption, analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
         </r>
       </text>
     </comment>
     <comment ref="H7" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
+          <t>Assumption, analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
         </r>
       </text>
     </comment>
     <comment ref="I7" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
+          <t>Assumption, analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
         </r>
       </text>
     </comment>
     <comment ref="J7" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
+          <t>Assumption, analyst judgment: AOV growth FY26E +6% (basket-mix + inflation; Q1-26 AOV +15% YoY on Snoonu mix), tapering to +3%.</t>
         </r>
       </text>
     </comment>
@@ -301,7 +301,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.24
-Open in Faheem — faheem://doc/fy24-ar/24
+Open in Faheem, faheem://doc/fy24-ar/24
 Actuals reported; orders×AOV ties within rounding.</t>
         </r>
       </text>
@@ -310,7 +310,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4
+Open in Faheem, faheem://doc/fy25-er/4
 Actuals reported; orders×AOV ties within rounding.</t>
         </r>
       </text>
@@ -319,7 +319,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4
+Open in Faheem, faheem://doc/fy25-er/4
 Actuals reported; orders×AOV ties within rounding.</t>
         </r>
       </text>
@@ -362,35 +362,35 @@
     <comment ref="F9" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5% — reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
+          <t>Assumption, analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5%, reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
         </r>
       </text>
     </comment>
     <comment ref="G9" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5% — reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
+          <t>Assumption, analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5%, reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
         </r>
       </text>
     </comment>
     <comment ref="H9" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5% — reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
+          <t>Assumption, analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5%, reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
         </r>
       </text>
     </comment>
     <comment ref="I9" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5% — reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
+          <t>Assumption, analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5%, reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
         </r>
       </text>
     </comment>
     <comment ref="J9" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5% — reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
+          <t>Assumption, analyst judgment: net-revenue monetisation (net revenue / GMV) eases from FY25's 32.1% to 31.0% in FY26E then holds at 30.5%, reflecting continued delivery-fee competition (KSA platform revenue fell 8.6% YoY in FY25) before stabilising.</t>
         </r>
       </text>
     </comment>
@@ -398,7 +398,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.5
-Open in Faheem — faheem://doc/fy24-ar/5</t>
+Open in Faheem, faheem://doc/fy24-ar/5</t>
         </r>
       </text>
     </comment>
@@ -406,7 +406,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -414,7 +414,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -457,7 +457,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.24
-Open in Faheem — faheem://doc/fy24-ar/24</t>
+Open in Faheem, faheem://doc/fy24-ar/24</t>
         </r>
       </text>
     </comment>
@@ -465,7 +465,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.5
-Open in Faheem — faheem://doc/fy24-ar/5</t>
+Open in Faheem, faheem://doc/fy24-ar/5</t>
         </r>
       </text>
     </comment>
@@ -473,7 +473,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.11
-Open in Faheem — faheem://doc/fy25-er/11</t>
+Open in Faheem, faheem://doc/fy25-er/11</t>
         </r>
       </text>
     </comment>
@@ -516,7 +516,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -524,7 +524,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.9
-Open in Faheem — faheem://doc/fy25-er/9</t>
+Open in Faheem, faheem://doc/fy25-er/9</t>
         </r>
       </text>
     </comment>
@@ -532,7 +532,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.9
-Open in Faheem — faheem://doc/fy25-er/9</t>
+Open in Faheem, faheem://doc/fy25-er/9</t>
         </r>
       </text>
     </comment>
@@ -540,7 +540,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.9
-Open in Faheem — faheem://doc/fy25-er/9</t>
+Open in Faheem, faheem://doc/fy25-er/9</t>
         </r>
       </text>
     </comment>
@@ -548,7 +548,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.9
-Open in Faheem — faheem://doc/fy25-er/9</t>
+Open in Faheem, faheem://doc/fy25-er/9</t>
         </r>
       </text>
     </comment>
@@ -628,35 +628,35 @@
     <comment ref="F6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds — a terminal margin at ~the FY24 peak plus modest leverage.</t>
+          <t>Assumption, analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds, a terminal margin at ~the FY24 peak plus modest leverage.</t>
         </r>
       </text>
     </comment>
     <comment ref="G6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds — a terminal margin at ~the FY24 peak plus modest leverage.</t>
+          <t>Assumption, analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds, a terminal margin at ~the FY24 peak plus modest leverage.</t>
         </r>
       </text>
     </comment>
     <comment ref="H6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds — a terminal margin at ~the FY24 peak plus modest leverage.</t>
+          <t>Assumption, analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds, a terminal margin at ~the FY24 peak plus modest leverage.</t>
         </r>
       </text>
     </comment>
     <comment ref="I6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds — a terminal margin at ~the FY24 peak plus modest leverage.</t>
+          <t>Assumption, analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds, a terminal margin at ~the FY24 peak plus modest leverage.</t>
         </r>
       </text>
     </comment>
     <comment ref="J6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds — a terminal margin at ~the FY24 peak plus modest leverage.</t>
+          <t>Assumption, analyst judgment: EBITDA margin path anchored to management's FY2026 guidance of SAR 200–220m adj. EBITDA (~7.5% on forecast revenue), recovering to 12.0% by FY30E as Q4-25 one-offs roll off, Snoonu (FY25 adj. EBITDA +SAR 53.7m, profitable) consolidates for a full year, and operating leverage builds, a terminal margin at ~the FY24 peak plus modest leverage.</t>
         </r>
       </text>
     </comment>
@@ -664,7 +664,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.5
-Open in Faheem — faheem://doc/fy24-ar/5</t>
+Open in Faheem, faheem://doc/fy24-ar/5</t>
         </r>
       </text>
     </comment>
@@ -672,7 +672,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -680,7 +680,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -688,7 +688,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.8
-Open in Faheem — faheem://doc/fy25-er/8</t>
+Open in Faheem, faheem://doc/fy25-er/8</t>
         </r>
       </text>
     </comment>
@@ -696,7 +696,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.8
-Open in Faheem — faheem://doc/fy25-er/8</t>
+Open in Faheem, faheem://doc/fy25-er/8</t>
         </r>
       </text>
     </comment>
@@ -739,7 +739,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Annual Report 2024, p.5
-Open in Faheem — faheem://doc/fy24-ar/5</t>
+Open in Faheem, faheem://doc/fy24-ar/5</t>
         </r>
       </text>
     </comment>
@@ -747,7 +747,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
@@ -755,56 +755,56 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q4 2025 Earnings Results, p.4
-Open in Faheem — faheem://doc/fy25-er/4</t>
+Open in Faheem, faheem://doc/fy25-er/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F10" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
+          <t>Assumption, analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
         </r>
       </text>
     </comment>
     <comment ref="G10" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
+          <t>Assumption, analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
         </r>
       </text>
     </comment>
     <comment ref="H10" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
+          <t>Assumption, analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
         </r>
       </text>
     </comment>
     <comment ref="I10" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
+          <t>Assumption, analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
         </r>
       </text>
     </comment>
     <comment ref="J10" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
+          <t>Assumption, analyst judgment: forecast net income simplified to EBIT×(1−zakat); net finance cost is ~nil given the net-cash balance sheet.</t>
         </r>
       </text>
     </comment>
     <comment ref="D15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: actual-year FCFF applies the same capex (2.5%) and ΔNWC (2.0%) assumptions to reported EBIT — capex is not separately disclosed, so this is an estimate, shown for continuity only (it does not feed the DCF).</t>
+          <t>Assumption, analyst judgment: actual-year FCFF applies the same capex (2.5%) and ΔNWC (2.0%) assumptions to reported EBIT, capex is not separately disclosed, so this is an estimate, shown for continuity only (it does not feed the DCF).</t>
         </r>
       </text>
     </comment>
     <comment ref="E15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: actual-year FCFF applies the same capex (2.5%) and ΔNWC (2.0%) assumptions to reported EBIT — capex is not separately disclosed, so this is an estimate, shown for continuity only (it does not feed the DCF).</t>
+          <t>Assumption, analyst judgment: actual-year FCFF applies the same capex (2.5%) and ΔNWC (2.0%) assumptions to reported EBIT, capex is not separately disclosed, so this is an estimate, shown for continuity only (it does not feed the DCF).</t>
         </r>
       </text>
     </comment>
@@ -847,7 +847,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.7
-Open in Faheem — faheem://doc/q1-26-fs/7</t>
+Open in Faheem, faheem://doc/q1-26-fs/7</t>
         </r>
       </text>
     </comment>
@@ -855,14 +855,14 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.4
-Open in Faheem — faheem://doc/q1-26-fs/4</t>
+Open in Faheem, faheem://doc/q1-26-fs/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F20" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: forecast cash rolled forward as prior-year cash + FCFF (no dividends/financing modelled — Jahez pays negligible dividends and is net-cash).</t>
+          <t>Assumption, analyst judgment: forecast cash rolled forward as prior-year cash + FCFF (no dividends/financing modelled, Jahez pays negligible dividends and is net-cash).</t>
         </r>
       </text>
     </comment>
@@ -870,14 +870,14 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.4
-Open in Faheem — faheem://doc/q1-26-fs/4</t>
+Open in Faheem, faheem://doc/q1-26-fs/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F21" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: interest-bearing debt and lease liabilities held flat at the FY25 audited level across the forecast (no disclosed amortisation schedule).</t>
+          <t>Assumption, analyst judgment: interest-bearing debt and lease liabilities held flat at the FY25 audited level across the forecast (no disclosed amortisation schedule).</t>
         </r>
       </text>
     </comment>
@@ -885,7 +885,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Q1 2026 Financial Statements, p.4
-Open in Faheem — faheem://doc/q1-26-fs/4</t>
+Open in Faheem, faheem://doc/q1-26-fs/4</t>
         </r>
       </text>
     </comment>
@@ -934,7 +934,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
@@ -942,7 +942,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
@@ -950,14 +950,14 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F6" authorId="0">
       <text>
         <r>
-          <t>n/a — no matched-period EV/GMV in sources</t>
+          <t>n/a, no matched-period EV/GMV in sources</t>
         </r>
       </text>
     </comment>
@@ -965,7 +965,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
@@ -973,7 +973,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
@@ -981,14 +981,14 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
     <comment ref="F8" authorId="0">
       <text>
         <r>
-          <t>n/a — no matched-period EV/GMV in sources</t>
+          <t>n/a, no matched-period EV/GMV in sources</t>
         </r>
       </text>
     </comment>
@@ -996,7 +996,7 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
@@ -1004,21 +1004,21 @@
       <text>
         <r>
           <t xml:space="preserve">Source: Market Data &amp; Comparables Snapshot, p.4
-Open in Faheem — faheem://doc/market-data-comps/4</t>
+Open in Faheem, faheem://doc/market-data-comps/4</t>
         </r>
       </text>
     </comment>
     <comment ref="E9" authorId="0">
       <text>
         <r>
-          <t>n/a — loss-making (TTM), P/E not meaningful</t>
+          <t>n/a, loss-making (TTM), P/E not meaningful</t>
         </r>
       </text>
     </comment>
     <comment ref="F9" authorId="0">
       <text>
         <r>
-          <t>n/a — no matched-period EV/GMV in sources</t>
+          <t>n/a, no matched-period EV/GMV in sources</t>
         </r>
       </text>
     </comment>
@@ -1056,35 +1056,35 @@
     <comment ref="C6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: scenario probabilities 25% bull / 50% base / 25% bear — analyst's central-case weighting.</t>
+          <t>Assumption, analyst judgment: scenario probabilities 25% bull / 50% base / 25% bear, analyst's central-case weighting.</t>
         </r>
       </text>
     </comment>
     <comment ref="D6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: scenario probabilities 25% bull / 50% base / 25% bear — analyst's central-case weighting.</t>
+          <t>Assumption, analyst judgment: scenario probabilities 25% bull / 50% base / 25% bear, analyst's central-case weighting.</t>
         </r>
       </text>
     </comment>
     <comment ref="E6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: scenario probabilities 25% bull / 50% base / 25% bear — analyst's central-case weighting.</t>
+          <t>Assumption, analyst judgment: scenario probabilities 25% bull / 50% base / 25% bear, analyst's central-case weighting.</t>
         </r>
       </text>
     </comment>
     <comment ref="H6" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull terminal growth 3.5%</t>
+          <t>Assumption, analyst judgment: bull terminal growth 3.5%</t>
         </r>
       </text>
     </comment>
     <comment ref="H7" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bear terminal growth 2.5%</t>
+          <t>Assumption, analyst judgment: bear terminal growth 2.5%</t>
         </r>
       </text>
     </comment>
@@ -1098,70 +1098,70 @@
     <comment ref="C13" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="D13" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="E13" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="F13" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="G13" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="C15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="D15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="E15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="F15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="G15" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
@@ -1175,77 +1175,77 @@
     <comment ref="E23" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: exit convention: the share price converges to intrinsic value at exit, and intrinsic value compounds at the cost of equity over the hold. IRR = (1+Ke)·(value/entry)^(1/years) − 1 — buying at fair value earns Ke; the discount to value is the additional annualised premium.</t>
+          <t>Assumption, analyst judgment: exit convention: the share price converges to intrinsic value at exit, and intrinsic value compounds at the cost of equity over the hold. IRR = (1+Ke)·(value/entry)^(1/years) − 1, buying at fair value earns Ke; the discount to value is the additional annualised premium.</t>
         </r>
       </text>
     </comment>
     <comment ref="C26" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="D26" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="E26" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="F26" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="G26" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="C28" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="D28" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="E28" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="F28" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="G28" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
@@ -1259,77 +1259,77 @@
     <comment ref="E36" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: exit convention: the share price converges to intrinsic value at exit, and intrinsic value compounds at the cost of equity over the hold. IRR = (1+Ke)·(value/entry)^(1/years) − 1 — buying at fair value earns Ke; the discount to value is the additional annualised premium.</t>
+          <t>Assumption, analyst judgment: exit convention: the share price converges to intrinsic value at exit, and intrinsic value compounds at the cost of equity over the hold. IRR = (1+Ke)·(value/entry)^(1/years) − 1, buying at fair value earns Ke; the discount to value is the additional annualised premium.</t>
         </r>
       </text>
     </comment>
     <comment ref="C39" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="D39" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="E39" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="F39" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="G39" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="C41" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="D41" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="E41" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="F41" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
     <comment ref="G41" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
+          <t>Assumption, analyst judgment: bull/bear apply parallel shifts to net-revenue growth (±~3–4pp/yr) and EBITDA margin (±1.5pp) with terminal growth of 3.5% / 2.5%; WACC is held constant to isolate the operating case.</t>
         </r>
       </text>
     </comment>
@@ -1343,91 +1343,91 @@
     <comment ref="E49" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: exit convention: the share price converges to intrinsic value at exit, and intrinsic value compounds at the cost of equity over the hold. IRR = (1+Ke)·(value/entry)^(1/years) − 1 — buying at fair value earns Ke; the discount to value is the additional annualised premium.</t>
+          <t>Assumption, analyst judgment: exit convention: the share price converges to intrinsic value at exit, and intrinsic value compounds at the cost of equity over the hold. IRR = (1+Ke)·(value/entry)^(1/years) − 1, buying at fair value earns Ke; the discount to value is the additional annualised premium.</t>
         </r>
       </text>
     </comment>
     <comment ref="C53" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: probability score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: probability score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="D53" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: impact score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: impact score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="C54" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: probability score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: probability score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="D54" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: impact score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: impact score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="C55" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: probability score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: probability score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="D55" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: impact score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: impact score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="C56" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: probability score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: probability score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="D56" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: impact score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: impact score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="C57" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: probability score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: probability score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="D57" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: impact score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: impact score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="C58" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: probability score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: probability score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
     <comment ref="D58" authorId="0">
       <text>
         <r>
-          <t>Assumption — analyst judgment: impact score 1–5 (analyst)</t>
+          <t>Assumption, analyst judgment: impact score 1–5 (analyst)</t>
         </r>
       </text>
     </comment>
@@ -1451,7 +1451,7 @@
     <t>Equity Research · Jahez International Company (Tadawul: 6017)</t>
   </si>
   <si>
-    <t>Rating (advisory only — the committee decides)</t>
+    <t>Rating (advisory only, the committee decides)</t>
   </si>
   <si>
     <t>Target price (DCF fair value)</t>
@@ -1472,7 +1472,7 @@
     <t>Hurdle rate (Lunar mandate)</t>
   </si>
   <si>
-    <t>Shariah screen</t>
+    <t>Compliance screen</t>
   </si>
   <si>
     <t>Composite risk (0–10)</t>
@@ -1481,10 +1481,10 @@
     <t>Weighted value / share</t>
   </si>
   <si>
-    <t>All figures are live formulas referencing the model tabs — target price = DCF!Value per share, upside = DCF, IRR &amp; weighted return = Scenarios &amp; Risk, Shariah = Shariah Screen. Advisory only: the Investment Committee decides. Prepared by Faheem for Lunar Investments, 12 Jul 2026. Not investment advice.</t>
-  </si>
-  <si>
-    <t>Lunar Investments · Jahez Group — Valuation Assumptions</t>
+    <t>All figures are live formulas referencing the model tabs, target price = DCF!Value per share, upside = DCF, IRR &amp; weighted return = Scenarios &amp; Risk, Compliance = Compliance Screen. Advisory only: the Investment Committee decides. Prepared by Faheem for Lunar Investments, 12 Jul 2026. Not investment advice.</t>
+  </si>
+  <si>
+    <t>Lunar Investments · Jahez Group, Valuation Assumptions</t>
   </si>
   <si>
     <t>Discount-rate build, terminal assumptions &amp; operating drivers</t>
@@ -1493,7 +1493,7 @@
     <t>1 · WACC build (discount rate)</t>
   </si>
   <si>
-    <t>Risk-free rate — Saudi 'Sah' sukuk proxy</t>
+    <t>Risk-free rate, Saudi 'Sah' sukuk proxy</t>
   </si>
   <si>
     <t>rate</t>
@@ -1502,10 +1502,10 @@
     <t>market-data-comps p.2</t>
   </si>
   <si>
-    <t>Equity risk premium — KSA total ERP (Damodaran)</t>
-  </si>
-  <si>
-    <t>Comp levered beta — DoorDash (DASH), 5Y</t>
+    <t>Equity risk premium, KSA total ERP (Damodaran)</t>
+  </si>
+  <si>
+    <t>Comp levered beta, DoorDash (DASH), 5Y</t>
   </si>
   <si>
     <t>x</t>
@@ -1514,10 +1514,10 @@
     <t>market-data-comps p.3</t>
   </si>
   <si>
-    <t>Comp levered beta — Delivery Hero (DHER), 5Y</t>
-  </si>
-  <si>
-    <t>Comp levered beta — Talabat (TALABAT)</t>
+    <t>Comp levered beta, Delivery Hero (DHER), 5Y</t>
+  </si>
+  <si>
+    <t>Comp levered beta, Talabat (TALABAT)</t>
   </si>
   <si>
     <t>n/a</t>
@@ -1526,13 +1526,13 @@
     <t>beta</t>
   </si>
   <si>
-    <t>Beta used — comp-set median</t>
+    <t>Beta used, comp-set median</t>
   </si>
   <si>
     <t>analyst judgment</t>
   </si>
   <si>
-    <t>Cost of equity — CAPM (rf + β × ERP)</t>
+    <t>Cost of equity, CAPM (rf + β × ERP)</t>
   </si>
   <si>
     <t>Cost-of-debt spread over rf</t>
@@ -1571,7 +1571,7 @@
     <t>SAR m</t>
   </si>
   <si>
-    <t>Interest-bearing debt — Islamic facilities (D)</t>
+    <t>Interest-bearing debt, Islamic facilities (D)</t>
   </si>
   <si>
     <t>q1-26-fs p.4</t>
@@ -1622,19 +1622,19 @@
     <t>4 · Operating drivers &amp; margins (analyst)</t>
   </si>
   <si>
-    <t>D&amp;A — % of net revenue</t>
-  </si>
-  <si>
-    <t>Capex — % of net revenue</t>
-  </si>
-  <si>
-    <t>ΔNWC — % of change in net revenue</t>
-  </si>
-  <si>
-    <t>Sourced cells (grey) carry the source document + page and a faheem:// deep-link into Faheem's viewer. Gold cells are labelled analyst assumptions — hover any cell for its full rationale.</t>
-  </si>
-  <si>
-    <t>Jahez Group — Revenue Drivers</t>
+    <t>D&amp;A, % of net revenue</t>
+  </si>
+  <si>
+    <t>Capex, % of net revenue</t>
+  </si>
+  <si>
+    <t>ΔNWC, % of change in net revenue</t>
+  </si>
+  <si>
+    <t>Sourced cells (grey) carry the source document + page and a faheem:// deep-link into Faheem's viewer. Gold cells are labelled analyst assumptions, hover any cell for its full rationale.</t>
+  </si>
+  <si>
+    <t>Jahez Group, Revenue Drivers</t>
   </si>
   <si>
     <t>Orders × AOV = GMV → monetisation → net revenue · FY23A–FY25A actuals, FY26E–FY30E driven</t>
@@ -1694,10 +1694,10 @@
     <t>FY2025 net-revenue segment split (SAR m)</t>
   </si>
   <si>
-    <t xml:space="preserve">  Platforms — KSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Platforms — Non-KSA</t>
+    <t xml:space="preserve">  Platforms, KSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Platforms, Non-KSA</t>
   </si>
   <si>
     <t xml:space="preserve">  Logistics</t>
@@ -1718,10 +1718,10 @@
     <t>Actuals (grey) sourced from Jahez filings; forecast columns (white) are formula-driven off the gold assumption cells. Segment revenues reconcile to the consolidated group total via inter-segment eliminations.</t>
   </si>
   <si>
-    <t>Jahez Group — Summary 3-Statement</t>
-  </si>
-  <si>
-    <t>P&amp;L · balance sheet · cash flow — FY23A–FY25A actual, FY26E–FY30E projected by formula</t>
+    <t>Jahez Group, Summary 3-Statement</t>
+  </si>
+  <si>
+    <t>P&amp;L · balance sheet · cash flow, FY23A–FY25A actual, FY26E–FY30E projected by formula</t>
   </si>
   <si>
     <t>Profit &amp; loss (SAR m)</t>
@@ -1772,7 +1772,7 @@
     <t>The projected FCFF row is the base of the DCF. Actual-year FCFF applies the same capex/ΔNWC assumptions to reported figures (capex is not separately disclosed) and is shown for continuity only.</t>
   </si>
   <si>
-    <t>Jahez Group — Discounted Cash Flow (FCFF)</t>
+    <t>Jahez Group, Discounted Cash Flow (FCFF)</t>
   </si>
   <si>
     <t>Explicit FY26E–FY30E PV + Gordon terminal value → enterprise value → equity bridge → value per share</t>
@@ -1832,28 +1832,28 @@
     <t>Every value is a live formula: PV factors read Assumptions!WACC, the terminal value uses Gordon growth, and the equity bridge subtracts debt &amp; leases and adds cash. Change any assumption and the whole chain recomputes.</t>
   </si>
   <si>
-    <t>Jahez Group — Sensitivity</t>
-  </si>
-  <si>
-    <t>Live formula grids (no data-table feature) — corners recompute from the DCF's own FCFF stream</t>
-  </si>
-  <si>
-    <t>Value per share (SAR) — WACC (→) × terminal growth (↓)</t>
+    <t>Jahez Group, Sensitivity</t>
+  </si>
+  <si>
+    <t>Live formula grids (no data-table feature), corners recompute from the DCF's own FCFF stream</t>
+  </si>
+  <si>
+    <t>Value per share (SAR), WACC (→) × terminal growth (↓)</t>
   </si>
   <si>
     <t>g \ WACC</t>
   </si>
   <si>
-    <t>FY30E Adj. EBITDA (SAR m) — GMV growth (→) × net-revenue rate (↓)</t>
+    <t>FY30E Adj. EBITDA (SAR m), GMV growth (→) × net-revenue rate (↓)</t>
   </si>
   <si>
     <t>take \ GMV g</t>
   </si>
   <si>
-    <t>Grid 1 cells hold the full DCF closed form — Σ FCFFₜ/(1+WACC)ᵗ + Gordon TV + net cash, all divided by shares — reading each column's WACC and each row's g live. The centre cell equals the DCF value per share exactly.</t>
-  </si>
-  <si>
-    <t>Jahez Group — Trading Comparables</t>
+    <t>Grid 1 cells hold the full DCF closed form, Σ FCFFₜ/(1+WACC)ᵗ + Gordon TV + net cash, all divided by shares, reading each column's WACC and each row's g live. The centre cell equals the DCF value per share exactly.</t>
+  </si>
+  <si>
+    <t>Jahez Group, Trading Comparables</t>
   </si>
   <si>
     <t>Sourced multiples → implied value per share · football field vs DCF · unsourced cells never filled</t>
@@ -1883,7 +1883,7 @@
     <t>Deliveroo (delisted)</t>
   </si>
   <si>
-    <t>Delisted — acquired by DoorDash 2 Oct 2025; no longer a standalone public comp</t>
+    <t>Delisted, acquired by DoorDash 2 Oct 2025; no longer a standalone public comp</t>
   </si>
   <si>
     <t>DoorDash (NASDAQ: DASH)</t>
@@ -1892,7 +1892,7 @@
     <t>Delivery Hero (ETR: DHER)</t>
   </si>
   <si>
-    <t>Implied value per share (SAR) — multiple × Jahez metric, bridged to equity</t>
+    <t>Implied value per share (SAR), multiple × Jahez metric, bridged to equity</t>
   </si>
   <si>
     <t>Jahez FY25A metric (SAR m / SAR)</t>
@@ -1907,25 +1907,25 @@
     <t xml:space="preserve">  Delivery Hero</t>
   </si>
   <si>
-    <t>Football field — implied value range vs DCF</t>
-  </si>
-  <si>
-    <t>Comps implied — minimum</t>
-  </si>
-  <si>
-    <t>Comps implied — median</t>
-  </si>
-  <si>
-    <t>Comps implied — maximum</t>
+    <t>Football field, implied value range vs DCF</t>
+  </si>
+  <si>
+    <t>Comps implied, minimum</t>
+  </si>
+  <si>
+    <t>Comps implied, median</t>
+  </si>
+  <si>
+    <t>Comps implied, maximum</t>
   </si>
   <si>
     <t>DCF value per share</t>
   </si>
   <si>
-    <t>The comp set is deliberately wide (single-market Talabat to scale-premium DoorDash) and trailing metrics are depressed by FY25 one-offs — treat comps as a sense-check on the DCF, not a standalone valuation. EV/GMV and Delivery Hero P/E are 'n/a — not sourced' and are never filled in.</t>
-  </si>
-  <si>
-    <t>Jahez Group — Scenarios &amp; Risk</t>
+    <t>The comp set is deliberately wide (single-market Talabat to scale-premium DoorDash) and trailing metrics are depressed by FY25 one-offs, treat comps as a sense-check on the DCF, not a standalone valuation. EV/GMV and Delivery Hero P/E are 'n/a, not sourced' and are never filled in.</t>
+  </si>
+  <si>
+    <t>Jahez Group, Scenarios &amp; Risk</t>
   </si>
   <si>
     <t>Bull / base / bear DCFs · IRR at entry vs 15% hurdle · scenario-weighted return · quantified risk register</t>
@@ -2078,7 +2078,7 @@
     <t>Bull/base/bear are full FCFF DCFs sharing the WACC build; only the operating drivers and terminal growth differ. IRR uses the documented exit convention (value compounds at Ke; price converges to value). Risk cites reference the Industry &amp; News Pack pages.</t>
   </si>
   <si>
-    <t>Jahez Group — Shariah Screen (AAOIFI-style)</t>
+    <t>Jahez Group, Compliance Screen (AAOIFI-style)</t>
   </si>
   <si>
     <t>Financial-ratio screens by formula from the balance sheet · pass/fail flags</t>
@@ -2111,16 +2111,16 @@
     <t>Cash &amp; interest-bearing securities / market cap</t>
   </si>
   <si>
-    <t>Cash only — interest-bearing securities not separately disclosed; screened on cash (&lt;33%)</t>
+    <t>Cash only, interest-bearing securities not separately disclosed; screened on cash (&lt;33%)</t>
   </si>
   <si>
     <t xml:space="preserve">  Memo: (debt + leases) / market cap</t>
   </si>
   <si>
-    <t>IFRS-16 leases included (stricter view) — still passes</t>
-  </si>
-  <si>
-    <t>Non-permissible income / total revenue</t>
+    <t>IFRS-16 leases included (stricter view), still passes</t>
+  </si>
+  <si>
+    <t>Non-eligible income / total revenue</t>
   </si>
   <si>
     <t>n/d</t>
@@ -2129,13 +2129,13 @@
     <t>PASS*</t>
   </si>
   <si>
-    <t>Not separately disclosed — screened via business-activity test (permissible food delivery/logistics; Islamic financing)</t>
-  </si>
-  <si>
-    <t>Overall Shariah screen</t>
-  </si>
-  <si>
-    <t>* Non-permissible income is not separately disclosed in the filings; per AAOIFI practice the position is screened via the business-activity test rather than a fabricated percentage. Leverage and liquidity screens both pass with wide headroom; the business is permissible and financed through Islamic facilities.</t>
+    <t>Not separately disclosed, screened via business-activity test (eligible food delivery/logistics; Islamic financing)</t>
+  </si>
+  <si>
+    <t>Overall Compliance screen</t>
+  </si>
+  <si>
+    <t>* Non-eligible income is not separately disclosed in the filings; per AAOIFI practice the position is screened via the business-activity test rather than a fabricated percentage. Leverage and liquidity screens both pass with wide headroom; the business is eligible and financed through Islamic facilities.</t>
   </si>
 </sst>
 </file>
@@ -3187,7 +3187,7 @@
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="str">
-        <f>'Shariah Screen'!E11</f>
+        <f>'Compliance Screen'!E11</f>
         <v>PASS</v>
       </c>
       <c r="C14" s="13">

</xml_diff>

<commit_message>
chore: checkpoint in-flight work from parallel sessions before demo-flow build
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/artifacts/jahez-valuation-model.xlsx
+++ b/public/artifacts/jahez-valuation-model.xlsx
@@ -2078,7 +2078,7 @@
     <t>Bull/base/bear are full FCFF DCFs sharing the WACC build; only the operating drivers and terminal growth differ. IRR uses the documented exit convention (value compounds at Ke; price converges to value). Risk cites reference the Industry &amp; News Pack pages.</t>
   </si>
   <si>
-    <t>Jahez Group, Compliance Screen (AAOIFI-style)</t>
+    <t>Jahez Group, Compliance Screen (Lunar IC Charter, SOCPA-endorsed IFRS figures)</t>
   </si>
   <si>
     <t>Financial-ratio screens by formula from the balance sheet · pass/fail flags</t>
@@ -2105,7 +2105,7 @@
     <t>Interest-bearing debt / market cap</t>
   </si>
   <si>
-    <t>Islamic facilities &amp; loans over market value of equity (AAOIFI leverage screen, &lt;33%)</t>
+    <t>Islamic facilities &amp; loans over market value of equity (IC Charter leverage screen, &lt;33%)</t>
   </si>
   <si>
     <t>Cash &amp; interest-bearing securities / market cap</t>
@@ -2135,7 +2135,7 @@
     <t>Overall Compliance screen</t>
   </si>
   <si>
-    <t>* Non-eligible income is not separately disclosed in the filings; per AAOIFI practice the position is screened via the business-activity test rather than a fabricated percentage. Leverage and liquidity screens both pass with wide headroom; the business is eligible and financed through Islamic facilities.</t>
+    <t>* Non-eligible income is not separately disclosed in the filings; per the IC Charter's methodology the position is screened via the business-activity test rather than a fabricated percentage. Leverage and liquidity screens both pass with wide headroom; the business is eligible and financed through Islamic facilities. Reporting basis: IAS 34 / IFRS as endorsed in the Kingdom of Saudi Arabia and SOCPA pronouncements (Q1 2026 FS, p.13, Statement of compliance).</t>
   </si>
 </sst>
 </file>

</xml_diff>